<commit_message>
ui ,register student option
</commit_message>
<xml_diff>
--- a/attendance.xlsx
+++ b/attendance.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -529,6 +529,51 @@
         <v>46100.46998833333</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>abhay kumar</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2305469</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>46100.58471149306</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>abhay kumar</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2305469</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="n">
+        <v>46100.89387671297</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>abhay kumar</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2305469</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="n">
+        <v>46100.95576215278</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Removed dataset from tracking
</commit_message>
<xml_diff>
--- a/attendance.xlsx
+++ b/attendance.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -589,6 +589,36 @@
         <v>46102.57130822917</v>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>abhay kumar</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2305469</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="n">
+        <v>46102.892490625</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>abhay kumar</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2305469</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="n">
+        <v>46102.94660894676</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
git hub connected to antigravity
</commit_message>
<xml_diff>
--- a/attendance.xlsx
+++ b/attendance.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -634,6 +634,36 @@
         <v>46103.57805119213</v>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>abhay kumar</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2305469</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="n">
+        <v>46103.8176146875</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>abhay kumar</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2305469</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="n">
+        <v>46109.52124631945</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
new datset etc added
</commit_message>
<xml_diff>
--- a/attendance.xlsx
+++ b/attendance.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -466,22 +466,22 @@
         </is>
       </c>
       <c r="C2" s="3" t="n">
-        <v>46098.89639478009</v>
+        <v>46115.44505700232</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>abhay kumar</t>
+          <t>gurpreet</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2305469</t>
+          <t>2305504</t>
         </is>
       </c>
       <c r="C3" s="3" t="n">
-        <v>46099.69219085648</v>
+        <v>46115.44660604167</v>
       </c>
     </row>
     <row r="4">
@@ -496,172 +496,67 @@
         </is>
       </c>
       <c r="C4" s="3" t="n">
-        <v>46100.45578342592</v>
+        <v>46115.48571886574</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>hanish choudhary</t>
+          <t>karamjot singh</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2305510</t>
+          <t>2305528</t>
         </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>46100.45827962963</v>
+        <v>46115.49613141204</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>gurpreet</t>
+          <t>aditya rana</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2305504</t>
+          <t>2305473</t>
         </is>
       </c>
       <c r="C6" s="3" t="n">
-        <v>46100.46998833333</v>
+        <v>46115.49875177084</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>abhay kumar</t>
+          <t>aditya rana</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2305469</t>
+          <t>2305473</t>
         </is>
       </c>
       <c r="C7" s="3" t="n">
-        <v>46100.58471149306</v>
+        <v>46115.63119957176</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>abhay kumar</t>
+          <t>hanish choudhary</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2305469</t>
+          <t>2305510</t>
         </is>
       </c>
       <c r="C8" s="3" t="n">
-        <v>46100.89387671297</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>abhay kumar</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>2305469</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="n">
-        <v>46100.95576215278</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>abhay kumar</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>2305469</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="n">
-        <v>46102.57130822917</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>abhay kumar</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>2305469</t>
-        </is>
-      </c>
-      <c r="C11" s="3" t="n">
-        <v>46102.892490625</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>abhay kumar</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>2305469</t>
-        </is>
-      </c>
-      <c r="C12" s="3" t="n">
-        <v>46102.94660894676</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>abhay kumar</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>2305469</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="n">
-        <v>46103.57805119213</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>abhay kumar</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>2305469</t>
-        </is>
-      </c>
-      <c r="C14" s="3" t="n">
-        <v>46103.8176146875</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>abhay kumar</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>2305469</t>
-        </is>
-      </c>
-      <c r="C15" s="3" t="n">
-        <v>46109.52124631945</v>
+        <v>46115.63120137731</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update backend and attendance file
</commit_message>
<xml_diff>
--- a/attendance.xlsx
+++ b/attendance.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -559,6 +559,21 @@
         <v>46115.63120137731</v>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>abhay kumar</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2305469</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="n">
+        <v>46155.5041453125</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>